<commit_message>
The numbers, taken back to back this time
Both sweeps in the same hour on the same idle machine, three passes of every scene. The branch comes out a couple of
percent quicker per frame in the median under llvmpipe, further ahead where there's a UI over the scene, and the two
scenes development never had (quickstart, pathtraced) sit on their own with nothing to compare to.
</commit_message>
<xml_diff>
--- a/docs/metrics/project-health-2-metrics.xlsx
+++ b/docs/metrics/project-health-2-metrics.xlsx
@@ -623,7 +623,7 @@
       <c r="B11" s="4" t="inlineStr"/>
       <c r="C11" s="4" t="inlineStr"/>
       <c r="D11" s="5" t="n">
-        <v>7.880541005394416</v>
+        <v>-2.15076813147552</v>
       </c>
     </row>
     <row r="12">
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>75.33333333333333</v>
+        <v>98</v>
       </c>
       <c r="C13" s="6" t="n">
         <v>103.1666666666667</v>
@@ -1035,40 +1035,40 @@
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>28.01666666666667</v>
+        <v>30.06666666666667</v>
       </c>
       <c r="C9" s="8" t="n">
         <v>30.77666666666667</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>9.851279000594889</v>
+        <v>2.361419068736145</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>36</v>
+        <v>33.33333333333334</v>
       </c>
       <c r="F9" s="8" t="n">
         <v>32.66666666666666</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>151.9</v>
+        <v>147.36</v>
       </c>
       <c r="H9" s="8" t="n">
         <v>121.64</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>0.238</v>
+        <v>0.286</v>
       </c>
       <c r="J9" s="8" t="n">
         <v>0.286</v>
       </c>
       <c r="K9" s="8" t="n">
-        <v>320.1666666666667</v>
+        <v>414.1666666666667</v>
       </c>
       <c r="L9" s="8" t="n">
         <v>379.6666666666667</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="N9" s="4" t="n">
         <v>70</v>
@@ -1089,22 +1089,22 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>29.30833333333333</v>
+        <v>31.22</v>
       </c>
       <c r="C10" s="8" t="n">
         <v>31.89333333333333</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>8.820017059994315</v>
+        <v>2.156737134315617</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>34.33333333333334</v>
+        <v>32</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>31.33333333333333</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>138.46</v>
+        <v>171.29</v>
       </c>
       <c r="H10" s="8" t="n">
         <v>164.76</v>
@@ -1116,13 +1116,13 @@
         <v>0.17</v>
       </c>
       <c r="K10" s="8" t="n">
-        <v>75.33333333333333</v>
+        <v>98</v>
       </c>
       <c r="L10" s="8" t="n">
         <v>115.8333333333333</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>112</v>
+        <v>131</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>120</v>
@@ -1143,40 +1143,40 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>38.26166666666667</v>
+        <v>42.03</v>
       </c>
       <c r="C11" s="8" t="n">
         <v>44.65166666666667</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>16.70078843054406</v>
+        <v>6.237608057736545</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>25.83333333333333</v>
+        <v>23.66666666666667</v>
       </c>
       <c r="F11" s="8" t="n">
         <v>22</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>201.6</v>
+        <v>211.54</v>
       </c>
       <c r="H11" s="8" t="n">
         <v>192.53</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>0.33</v>
+        <v>0.418</v>
       </c>
       <c r="J11" s="8" t="n">
         <v>0.436</v>
       </c>
       <c r="K11" s="8" t="n">
-        <v>353</v>
+        <v>487</v>
       </c>
       <c r="L11" s="8" t="n">
         <v>526</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="N11" s="4" t="n">
         <v>150</v>
@@ -1197,34 +1197,34 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>35.35333333333333</v>
+        <v>39.02333333333333</v>
       </c>
       <c r="C12" s="8" t="n">
         <v>37.415</v>
       </c>
-      <c r="D12" s="9" t="n">
-        <v>5.831604752027157</v>
+      <c r="D12" s="10" t="n">
+        <v>-4.121465789698473</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>28.66666666666667</v>
+        <v>25.83333333333333</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>27.16666666666667</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>149.04</v>
+        <v>147.52</v>
       </c>
       <c r="H12" s="8" t="n">
         <v>135.27</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>0.2</v>
+        <v>0.252</v>
       </c>
       <c r="J12" s="8" t="n">
         <v>0.242</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>3528.333333333333</v>
+        <v>4508.833333333333</v>
       </c>
       <c r="L12" s="8" t="n">
         <v>3897.666666666667</v>
@@ -1251,40 +1251,40 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>28.53666666666667</v>
+        <v>31.065</v>
       </c>
       <c r="C13" s="8" t="n">
         <v>32.14333333333333</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>12.6387104310244</v>
+        <v>3.4712162669671</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>35.16666666666666</v>
+        <v>32.5</v>
       </c>
       <c r="F13" s="8" t="n">
         <v>31.33333333333333</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>150.46</v>
+        <v>153.81</v>
       </c>
       <c r="H13" s="8" t="n">
         <v>126.68</v>
       </c>
       <c r="I13" s="8" t="n">
-        <v>0.102</v>
+        <v>0.126</v>
       </c>
       <c r="J13" s="8" t="n">
         <v>0.122</v>
       </c>
       <c r="K13" s="8" t="n">
-        <v>66.33333333333333</v>
+        <v>79.5</v>
       </c>
       <c r="L13" s="8" t="n">
         <v>117.8333333333333</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="N13" s="4" t="n">
         <v>90</v>
@@ -1305,40 +1305,40 @@
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>21.575</v>
+        <v>24.55666666666667</v>
       </c>
       <c r="C14" s="8" t="n">
         <v>22.79</v>
       </c>
-      <c r="D14" s="9" t="n">
-        <v>5.631517960602548</v>
+      <c r="D14" s="10" t="n">
+        <v>-7.194244604316557</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>46.5</v>
+        <v>40.66666666666666</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>44.33333333333334</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>168.87</v>
+        <v>207.38</v>
       </c>
       <c r="H14" s="8" t="n">
         <v>148.49</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>0.19</v>
+        <v>0.222</v>
       </c>
       <c r="J14" s="8" t="n">
         <v>0.212</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>49.5</v>
+        <v>54</v>
       </c>
       <c r="L14" s="8" t="n">
         <v>49</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>137</v>
+        <v>172</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>112</v>
@@ -1367,40 +1367,40 @@
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>127.3</v>
+        <v>132.334</v>
       </c>
       <c r="C15" s="8" t="n">
         <v>133.556</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>4.914375490966233</v>
+        <v>0.9234210407000532</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>6.833333333333333</v>
+        <v>6.4</v>
       </c>
       <c r="F15" s="8" t="n">
         <v>7</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>532.77</v>
+        <v>538.26</v>
       </c>
       <c r="H15" s="8" t="n">
         <v>512.63</v>
       </c>
       <c r="I15" s="8" t="n">
-        <v>0.092</v>
+        <v>0.108</v>
       </c>
       <c r="J15" s="8" t="n">
         <v>0.112</v>
       </c>
       <c r="K15" s="8" t="n">
-        <v>82472.16666666667</v>
+        <v>85329.33333333333</v>
       </c>
       <c r="L15" s="8" t="n">
         <v>90695.83333333333</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>466</v>
+        <v>478</v>
       </c>
       <c r="N15" s="4" t="n">
         <v>442</v>
@@ -1421,28 +1421,28 @@
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>12.58333333333333</v>
+        <v>13.74833333333333</v>
       </c>
       <c r="C16" s="8" t="n">
         <v>12.49166666666667</v>
       </c>
       <c r="D16" s="10" t="n">
-        <v>-0.7284768211920539</v>
+        <v>-9.140501879015634</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>80</v>
+        <v>72.83333333333333</v>
       </c>
       <c r="F16" s="8" t="n">
         <v>80.5</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>22.96</v>
+        <v>28.5</v>
       </c>
       <c r="H16" s="8" t="n">
         <v>20.53</v>
       </c>
       <c r="I16" s="8" t="n">
-        <v>0.052</v>
+        <v>0.062</v>
       </c>
       <c r="J16" s="8" t="n">
         <v>0.07200000000000001</v>
@@ -1454,7 +1454,7 @@
         <v>48</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="N16" s="4" t="n">
         <v>23</v>
@@ -1475,40 +1475,40 @@
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>118.83</v>
+        <v>129.354</v>
       </c>
       <c r="C17" s="8" t="n">
         <v>126.606</v>
       </c>
-      <c r="D17" s="9" t="n">
-        <v>6.543802070184306</v>
+      <c r="D17" s="10" t="n">
+        <v>-2.124402801614178</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F17" s="8" t="n">
         <v>7.8</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>329.59</v>
+        <v>383.19</v>
       </c>
       <c r="H17" s="8" t="n">
         <v>352.76</v>
       </c>
       <c r="I17" s="8" t="n">
-        <v>0.078</v>
+        <v>0.09</v>
       </c>
       <c r="J17" s="8" t="n">
         <v>0.118</v>
       </c>
       <c r="K17" s="8" t="n">
-        <v>32420.4</v>
+        <v>41779</v>
       </c>
       <c r="L17" s="8" t="n">
         <v>40441</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>221</v>
+        <v>250</v>
       </c>
       <c r="N17" s="4" t="n">
         <v>224</v>
@@ -1529,40 +1529,40 @@
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>19.59833333333333</v>
+        <v>21.96166666666667</v>
       </c>
       <c r="C18" s="8" t="n">
         <v>22.20166666666667</v>
       </c>
       <c r="D18" s="9" t="n">
-        <v>13.28344246959776</v>
+        <v>1.092813235182524</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>51.33333333333334</v>
+        <v>45.83333333333334</v>
       </c>
       <c r="F18" s="8" t="n">
         <v>45</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>29.29</v>
+        <v>125.81</v>
       </c>
       <c r="H18" s="8" t="n">
         <v>111.54</v>
       </c>
       <c r="I18" s="8" t="n">
-        <v>0.054</v>
+        <v>0.062</v>
       </c>
       <c r="J18" s="8" t="n">
         <v>0.068</v>
       </c>
       <c r="K18" s="8" t="n">
-        <v>61.5</v>
+        <v>49</v>
       </c>
       <c r="L18" s="8" t="n">
         <v>50</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="N18" s="4" t="n">
         <v>77</v>
@@ -1583,40 +1583,40 @@
         </is>
       </c>
       <c r="B19" s="8" t="n">
-        <v>20.00166666666667</v>
+        <v>21.565</v>
       </c>
       <c r="C19" s="8" t="n">
         <v>21.63</v>
       </c>
-      <c r="D19" s="9" t="n">
-        <v>8.140988250979069</v>
+      <c r="D19" s="8" t="n">
+        <v>0.301414328773465</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>49.83333333333334</v>
+        <v>46.5</v>
       </c>
       <c r="F19" s="8" t="n">
         <v>46.16666666666666</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>41.18</v>
+        <v>110.57</v>
       </c>
       <c r="H19" s="8" t="n">
         <v>111.12</v>
       </c>
       <c r="I19" s="8" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.102</v>
       </c>
       <c r="J19" s="8" t="n">
         <v>0.1</v>
       </c>
       <c r="K19" s="8" t="n">
-        <v>48.5</v>
+        <v>49</v>
       </c>
       <c r="L19" s="8" t="n">
         <v>48.5</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="N19" s="4" t="n">
         <v>50</v>
@@ -1637,40 +1637,40 @@
         </is>
       </c>
       <c r="B20" s="8" t="n">
-        <v>30.92666666666667</v>
+        <v>33.37333333333333</v>
       </c>
       <c r="C20" s="8" t="n">
         <v>27.20166666666667</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>-12.04462168570812</v>
+        <v>-18.49280862964443</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>32.16666666666666</v>
+        <v>29.83333333333333</v>
       </c>
       <c r="F20" s="8" t="n">
         <v>36.5</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>335.3</v>
+        <v>364.6</v>
       </c>
       <c r="H20" s="8" t="n">
         <v>208.47</v>
       </c>
       <c r="I20" s="8" t="n">
-        <v>0.098</v>
+        <v>0.12</v>
       </c>
       <c r="J20" s="8" t="n">
         <v>0.126</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>328.3333333333333</v>
+        <v>552.8333333333334</v>
       </c>
       <c r="L20" s="8" t="n">
         <v>103.1666666666667</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>301</v>
+        <v>332</v>
       </c>
       <c r="N20" s="4" t="n">
         <v>172</v>
@@ -1691,40 +1691,40 @@
         </is>
       </c>
       <c r="B21" s="8" t="n">
-        <v>19.58666666666667</v>
+        <v>23.25666666666667</v>
       </c>
       <c r="C21" s="8" t="n">
         <v>21.50833333333333</v>
       </c>
-      <c r="D21" s="9" t="n">
-        <v>9.811095983662357</v>
+      <c r="D21" s="10" t="n">
+        <v>-7.517557689551389</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>51.16666666666666</v>
+        <v>43.16666666666666</v>
       </c>
       <c r="F21" s="8" t="n">
         <v>46.66666666666666</v>
       </c>
       <c r="G21" s="8" t="n">
-        <v>145.33</v>
+        <v>141.05</v>
       </c>
       <c r="H21" s="8" t="n">
         <v>128.59</v>
       </c>
       <c r="I21" s="8" t="n">
-        <v>0.102</v>
+        <v>0.148</v>
       </c>
       <c r="J21" s="8" t="n">
         <v>0.136</v>
       </c>
       <c r="K21" s="8" t="n">
-        <v>49.66666666666666</v>
+        <v>51</v>
       </c>
       <c r="L21" s="8" t="n">
         <v>52.83333333333334</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="N21" s="4" t="n">
         <v>94</v>
@@ -1745,40 +1745,40 @@
         </is>
       </c>
       <c r="B22" s="8" t="n">
-        <v>20.555</v>
+        <v>21.86333333333333</v>
       </c>
       <c r="C22" s="8" t="n">
         <v>21.25666666666667</v>
       </c>
-      <c r="D22" s="9" t="n">
-        <v>3.41360577312901</v>
+      <c r="D22" s="10" t="n">
+        <v>-2.774813233724648</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>49</v>
+        <v>46.16666666666666</v>
       </c>
       <c r="F22" s="8" t="n">
         <v>47</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>188.18</v>
+        <v>199.12</v>
       </c>
       <c r="H22" s="8" t="n">
         <v>158.88</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>0.186</v>
+        <v>0.212</v>
       </c>
       <c r="J22" s="8" t="n">
         <v>0.194</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>49.16666666666666</v>
+        <v>50.16666666666666</v>
       </c>
       <c r="L22" s="8" t="n">
         <v>49.83333333333334</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>152</v>
+        <v>171</v>
       </c>
       <c r="N22" s="4" t="n">
         <v>125</v>
@@ -1799,40 +1799,40 @@
         </is>
       </c>
       <c r="B23" s="8" t="n">
-        <v>20.68833333333333</v>
+        <v>23.325</v>
       </c>
       <c r="C23" s="8" t="n">
         <v>22.82333333333333</v>
       </c>
-      <c r="D23" s="9" t="n">
-        <v>10.31982598888263</v>
+      <c r="D23" s="10" t="n">
+        <v>-2.15076813147552</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>48.33333333333334</v>
+        <v>43.33333333333334</v>
       </c>
       <c r="F23" s="8" t="n">
         <v>44.5</v>
       </c>
       <c r="G23" s="8" t="n">
-        <v>33.99</v>
+        <v>34.6</v>
       </c>
       <c r="H23" s="8" t="n">
         <v>45.67</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>0.09</v>
+        <v>0.11</v>
       </c>
       <c r="J23" s="8" t="n">
         <v>0.112</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>86.83333333333333</v>
+        <v>55.33333333333334</v>
       </c>
       <c r="L23" s="8" t="n">
         <v>56.16666666666666</v>
       </c>
       <c r="M23" s="4" t="n">
-        <v>88</v>
+        <v>125</v>
       </c>
       <c r="N23" s="4" t="n">
         <v>84</v>
@@ -1853,40 +1853,40 @@
         </is>
       </c>
       <c r="B24" s="8" t="n">
-        <v>28.728</v>
+        <v>31.885</v>
       </c>
       <c r="C24" s="8" t="n">
         <v>31.47666666666667</v>
       </c>
-      <c r="D24" s="9" t="n">
-        <v>9.567901234567895</v>
+      <c r="D24" s="10" t="n">
+        <v>-1.280643980973295</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>34.8</v>
+        <v>31.16666666666667</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>31.5</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>100.4</v>
+        <v>110.38</v>
       </c>
       <c r="H24" s="8" t="n">
         <v>91.89</v>
       </c>
       <c r="I24" s="8" t="n">
-        <v>0.142</v>
+        <v>0.172</v>
       </c>
       <c r="J24" s="8" t="n">
         <v>0.178</v>
       </c>
       <c r="K24" s="8" t="n">
-        <v>74.33333333333333</v>
+        <v>100.6666666666667</v>
       </c>
       <c r="L24" s="8" t="n">
         <v>74.66666666666667</v>
       </c>
       <c r="M24" s="4" t="n">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="N24" s="4" t="n">
         <v>47</v>
@@ -1915,40 +1915,40 @@
         </is>
       </c>
       <c r="B25" s="8" t="n">
-        <v>24.05166666666667</v>
+        <v>25.725</v>
       </c>
       <c r="C25" s="8" t="n">
         <v>25.97666666666667</v>
       </c>
       <c r="D25" s="9" t="n">
-        <v>8.003603353890933</v>
+        <v>0.9782960803368906</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>41.66666666666666</v>
+        <v>39</v>
       </c>
       <c r="F25" s="8" t="n">
         <v>38.5</v>
       </c>
       <c r="G25" s="8" t="n">
-        <v>100.31</v>
+        <v>96.14</v>
       </c>
       <c r="H25" s="8" t="n">
         <v>108.63</v>
       </c>
       <c r="I25" s="8" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.096</v>
       </c>
       <c r="J25" s="8" t="n">
         <v>0.104</v>
       </c>
       <c r="K25" s="8" t="n">
-        <v>60.5</v>
+        <v>64.66666666666667</v>
       </c>
       <c r="L25" s="8" t="n">
         <v>68.83333333333333</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="N25" s="4" t="n">
         <v>35</v>
@@ -1969,40 +1969,40 @@
         </is>
       </c>
       <c r="B26" s="8" t="n">
-        <v>22.23166666666667</v>
+        <v>25.16166666666667</v>
       </c>
       <c r="C26" s="8" t="n">
         <v>23.98333333333333</v>
       </c>
-      <c r="D26" s="9" t="n">
-        <v>7.879151360671724</v>
+      <c r="D26" s="10" t="n">
+        <v>-4.6830496125058</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>45.33333333333334</v>
+        <v>39.83333333333334</v>
       </c>
       <c r="F26" s="8" t="n">
         <v>42.16666666666666</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>102.46</v>
+        <v>117.64</v>
       </c>
       <c r="H26" s="8" t="n">
         <v>108.59</v>
       </c>
       <c r="I26" s="8" t="n">
-        <v>0.148</v>
+        <v>0.156</v>
       </c>
       <c r="J26" s="8" t="n">
         <v>0.174</v>
       </c>
       <c r="K26" s="8" t="n">
-        <v>54</v>
+        <v>60.5</v>
       </c>
       <c r="L26" s="8" t="n">
         <v>62</v>
       </c>
       <c r="M26" s="4" t="n">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="N26" s="4" t="n">
         <v>60</v>
@@ -2023,40 +2023,40 @@
         </is>
       </c>
       <c r="B27" s="8" t="n">
-        <v>22.86666666666667</v>
+        <v>24.56666666666667</v>
       </c>
       <c r="C27" s="8" t="n">
         <v>23.85833333333333</v>
       </c>
-      <c r="D27" s="9" t="n">
-        <v>4.336734693877553</v>
+      <c r="D27" s="10" t="n">
+        <v>-2.88331071913161</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F27" s="8" t="n">
         <v>42.33333333333334</v>
       </c>
       <c r="G27" s="8" t="n">
-        <v>136.65</v>
+        <v>146.25</v>
       </c>
       <c r="H27" s="8" t="n">
         <v>113.3</v>
       </c>
       <c r="I27" s="8" t="n">
-        <v>0.126</v>
+        <v>0.14</v>
       </c>
       <c r="J27" s="8" t="n">
         <v>0.142</v>
       </c>
       <c r="K27" s="8" t="n">
-        <v>76.33333333333333</v>
+        <v>110.8333333333333</v>
       </c>
       <c r="L27" s="8" t="n">
         <v>80.16666666666667</v>
       </c>
       <c r="M27" s="4" t="n">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="N27" s="4" t="n">
         <v>83</v>
@@ -2077,40 +2077,40 @@
         </is>
       </c>
       <c r="B28" s="8" t="n">
-        <v>21.31833333333334</v>
+        <v>23.90666666666667</v>
       </c>
       <c r="C28" s="8" t="n">
         <v>22.99833333333333</v>
       </c>
-      <c r="D28" s="9" t="n">
-        <v>7.880541005394416</v>
+      <c r="D28" s="10" t="n">
+        <v>-3.799498047964298</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>47.16666666666666</v>
+        <v>42</v>
       </c>
       <c r="F28" s="8" t="n">
         <v>43.5</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>146.82</v>
+        <v>150.41</v>
       </c>
       <c r="H28" s="8" t="n">
         <v>125.92</v>
       </c>
       <c r="I28" s="8" t="n">
-        <v>0.118</v>
+        <v>0.144</v>
       </c>
       <c r="J28" s="8" t="n">
         <v>0.148</v>
       </c>
       <c r="K28" s="8" t="n">
-        <v>221.1666666666667</v>
+        <v>337.3333333333333</v>
       </c>
       <c r="L28" s="8" t="n">
         <v>341</v>
       </c>
       <c r="M28" s="4" t="n">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="N28" s="4" t="n">
         <v>91</v>
@@ -2131,40 +2131,40 @@
         </is>
       </c>
       <c r="B29" s="8" t="n">
-        <v>24.98666666666666</v>
+        <v>26.98666666666667</v>
       </c>
       <c r="C29" s="8" t="n">
         <v>25.75833333333333</v>
       </c>
-      <c r="D29" s="9" t="n">
-        <v>3.088313767342589</v>
+      <c r="D29" s="10" t="n">
+        <v>-4.551630434782616</v>
       </c>
       <c r="E29" s="8" t="n">
-        <v>41.16666666666666</v>
+        <v>37.33333333333334</v>
       </c>
       <c r="F29" s="8" t="n">
         <v>39.33333333333334</v>
       </c>
       <c r="G29" s="8" t="n">
-        <v>144.06</v>
+        <v>160.52</v>
       </c>
       <c r="H29" s="8" t="n">
         <v>139.95</v>
       </c>
       <c r="I29" s="8" t="n">
-        <v>0.192</v>
+        <v>0.226</v>
       </c>
       <c r="J29" s="8" t="n">
         <v>0.222</v>
       </c>
       <c r="K29" s="8" t="n">
-        <v>76849</v>
+        <v>85010.83333333333</v>
       </c>
       <c r="L29" s="8" t="n">
         <v>74821.83333333333</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>112</v>
+        <v>132</v>
       </c>
       <c r="N29" s="4" t="n">
         <v>103</v>

</xml_diff>